<commit_message>
Informe día 9, por la tarde
Solo gastamos los intentos de la IA flow de google labs, ademas de seguir un poco con el informe, entre otras cosas.
</commit_message>
<xml_diff>
--- a/registro_estancias.xlsx
+++ b/registro_estancias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frang\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357A8F1B-0E28-455F-8FAB-250559300437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DCBC7F6-2C98-449C-844C-9674307F1C94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="21">
   <si>
     <t>Alumno/a:</t>
   </si>
@@ -95,6 +95,12 @@
   </si>
   <si>
     <t>5:30 h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gastar los intentos que tenemos con Flow </t>
+  </si>
+  <si>
+    <t>2:00 h</t>
   </si>
 </sst>
 </file>
@@ -265,6 +271,18 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="14" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -277,18 +295,6 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Énfasis1" xfId="2" builtinId="29"/>
@@ -296,65 +302,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="22">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -562,6 +509,65 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -577,45 +583,45 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0BDF8D52-2453-4F9C-ACB9-A42D249CFCDF}" name="Fecha" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{04B31198-F76D-4FF5-9268-5FDFE4ECEBE2}" name="Hora inicio" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{DDD0E146-15E7-4D7C-B06E-B38DE0296A38}" name="Hora fin" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{F1A9F247-B63D-4C25-9111-14F13A0959C9}" name="Tareas realizadas" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{32907A34-0575-4F46-A5D0-8BFC39ACFB84}" name="Tiempo dedicado (h)" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{A6ABF540-9F00-4B21-9CD1-F5694FC959C9}" name="Lugar de realización" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{0BDF8D52-2453-4F9C-ACB9-A42D249CFCDF}" name="Fecha" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{04B31198-F76D-4FF5-9268-5FDFE4ECEBE2}" name="Hora inicio" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{DDD0E146-15E7-4D7C-B06E-B38DE0296A38}" name="Hora fin" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{F1A9F247-B63D-4C25-9111-14F13A0959C9}" name="Tareas realizadas" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{32907A34-0575-4F46-A5D0-8BFC39ACFB84}" name="Tiempo dedicado (h)" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{A6ABF540-9F00-4B21-9CD1-F5694FC959C9}" name="Lugar de realización" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="13" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{6717099B-BCF7-48F1-8C12-2FB104043E34}" name="Fecha" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{62A61D49-49F7-40AD-B517-D821200346E1}" name="Hora inicio" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{0EC89713-22B4-4357-96FB-DDBA8AAFD4E2}" name="Hora fin" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{1535F3D9-2D46-4B00-AC9D-A3B5A1FAE726}" name="Tareas realizadas" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{5C84EBA8-F84D-40E8-8B50-A63C5489A5D3}" name="Tiempo dedicado (h)" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{A113B472-3061-44DC-830B-0CB7CF97CD1F}" name="Lugar de realización" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{6717099B-BCF7-48F1-8C12-2FB104043E34}" name="Fecha" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{62A61D49-49F7-40AD-B517-D821200346E1}" name="Hora inicio" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{0EC89713-22B4-4357-96FB-DDBA8AAFD4E2}" name="Hora fin" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{1535F3D9-2D46-4B00-AC9D-A3B5A1FAE726}" name="Tareas realizadas" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{5C84EBA8-F84D-40E8-8B50-A63C5489A5D3}" name="Tiempo dedicado (h)" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{A113B472-3061-44DC-830B-0CB7CF97CD1F}" name="Lugar de realización" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="21" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{08C5D867-C4F7-42FE-B57C-F663CFF2AF17}" name="Fecha" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{C94CC689-C9E6-48B0-9B66-144C47C374AC}" name="Hora inicio" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{257A2ACB-E90D-4206-9538-AE9CCA80B025}" name="Hora fin" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{D70305DF-1893-438D-A18F-E5A3143BA874}" name="Tareas realizadas" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{C97A83D8-08D8-4681-88A5-C08F198EFF87}" name="Tiempo dedicado (h)" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{1089505E-D1F6-49DF-BAB1-9822A7A38FB6}" name="Lugar de realización" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{08C5D867-C4F7-42FE-B57C-F663CFF2AF17}" name="Fecha" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{C94CC689-C9E6-48B0-9B66-144C47C374AC}" name="Hora inicio" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{257A2ACB-E90D-4206-9538-AE9CCA80B025}" name="Hora fin" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{D70305DF-1893-438D-A18F-E5A3143BA874}" name="Tareas realizadas" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{C97A83D8-08D8-4681-88A5-C08F198EFF87}" name="Tiempo dedicado (h)" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{1089505E-D1F6-49DF-BAB1-9822A7A38FB6}" name="Lugar de realización" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -924,13 +930,13 @@
       <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B3" s="9"/>
@@ -939,13 +945,13 @@
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="N5" s="8" t="s">
@@ -999,9 +1005,24 @@
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="11"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
+      <c r="B8" s="2">
+        <v>46121</v>
+      </c>
+      <c r="C8" s="12">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D8" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9" s="11"/>
@@ -1255,13 +1276,13 @@
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B3" s="4"/>
@@ -1270,13 +1291,13 @@
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="N5" s="1" t="s">
@@ -1330,9 +1351,24 @@
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="2"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
+      <c r="B8" s="2">
+        <v>46121</v>
+      </c>
+      <c r="C8" s="12">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D8" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9" s="2"/>
@@ -1586,13 +1622,13 @@
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B3" s="4"/>
@@ -1601,13 +1637,13 @@
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="N5" s="1" t="s">
@@ -1661,9 +1697,24 @@
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="2"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
+      <c r="B8" s="2">
+        <v>46121</v>
+      </c>
+      <c r="C8" s="12">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D8" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9" s="2"/>

</xml_diff>

<commit_message>
Reporte de asistencias día 14
</commit_message>
<xml_diff>
--- a/registro_estancias.xlsx
+++ b/registro_estancias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frang\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C84C2FED-EC60-454B-A5D9-318FF6039733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA3D0088-DEE6-4554-B840-9FF23B022262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nombre1" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="27">
   <si>
     <t>Alumno/a:</t>
   </si>
@@ -113,6 +113,12 @@
   </si>
   <si>
     <t>Creacion del video y la redaccion del guión</t>
+  </si>
+  <si>
+    <t>Seguir con el guión y creación del informe</t>
+  </si>
+  <si>
+    <t>Gastar intentos de la IA, juntando algunos</t>
   </si>
 </sst>
 </file>
@@ -284,18 +290,6 @@
     <xf numFmtId="14" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -308,6 +302,18 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Énfasis1" xfId="2" builtinId="29"/>
@@ -315,6 +321,65 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="22">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -523,65 +588,6 @@
         <scheme val="minor"/>
       </font>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -596,45 +602,45 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0BDF8D52-2453-4F9C-ACB9-A42D249CFCDF}" name="Fecha" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{04B31198-F76D-4FF5-9268-5FDFE4ECEBE2}" name="Hora inicio" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{DDD0E146-15E7-4D7C-B06E-B38DE0296A38}" name="Hora fin" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{F1A9F247-B63D-4C25-9111-14F13A0959C9}" name="Tareas realizadas" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{32907A34-0575-4F46-A5D0-8BFC39ACFB84}" name="Tiempo dedicado (h)" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{A6ABF540-9F00-4B21-9CD1-F5694FC959C9}" name="Lugar de realización" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{0BDF8D52-2453-4F9C-ACB9-A42D249CFCDF}" name="Fecha" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{04B31198-F76D-4FF5-9268-5FDFE4ECEBE2}" name="Hora inicio" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{DDD0E146-15E7-4D7C-B06E-B38DE0296A38}" name="Hora fin" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{F1A9F247-B63D-4C25-9111-14F13A0959C9}" name="Tareas realizadas" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{32907A34-0575-4F46-A5D0-8BFC39ACFB84}" name="Tiempo dedicado (h)" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{A6ABF540-9F00-4B21-9CD1-F5694FC959C9}" name="Lugar de realización" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="13" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{6717099B-BCF7-48F1-8C12-2FB104043E34}" name="Fecha" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{62A61D49-49F7-40AD-B517-D821200346E1}" name="Hora inicio" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{0EC89713-22B4-4357-96FB-DDBA8AAFD4E2}" name="Hora fin" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{1535F3D9-2D46-4B00-AC9D-A3B5A1FAE726}" name="Tareas realizadas" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{5C84EBA8-F84D-40E8-8B50-A63C5489A5D3}" name="Tiempo dedicado (h)" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{A113B472-3061-44DC-830B-0CB7CF97CD1F}" name="Lugar de realización" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{6717099B-BCF7-48F1-8C12-2FB104043E34}" name="Fecha" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{62A61D49-49F7-40AD-B517-D821200346E1}" name="Hora inicio" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{0EC89713-22B4-4357-96FB-DDBA8AAFD4E2}" name="Hora fin" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{1535F3D9-2D46-4B00-AC9D-A3B5A1FAE726}" name="Tareas realizadas" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{5C84EBA8-F84D-40E8-8B50-A63C5489A5D3}" name="Tiempo dedicado (h)" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{A113B472-3061-44DC-830B-0CB7CF97CD1F}" name="Lugar de realización" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="21" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{08C5D867-C4F7-42FE-B57C-F663CFF2AF17}" name="Fecha" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{C94CC689-C9E6-48B0-9B66-144C47C374AC}" name="Hora inicio" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{257A2ACB-E90D-4206-9538-AE9CCA80B025}" name="Hora fin" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{D70305DF-1893-438D-A18F-E5A3143BA874}" name="Tareas realizadas" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{C97A83D8-08D8-4681-88A5-C08F198EFF87}" name="Tiempo dedicado (h)" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{1089505E-D1F6-49DF-BAB1-9822A7A38FB6}" name="Lugar de realización" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{08C5D867-C4F7-42FE-B57C-F663CFF2AF17}" name="Fecha" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{C94CC689-C9E6-48B0-9B66-144C47C374AC}" name="Hora inicio" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{257A2ACB-E90D-4206-9538-AE9CCA80B025}" name="Hora fin" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{D70305DF-1893-438D-A18F-E5A3143BA874}" name="Tareas realizadas" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{C97A83D8-08D8-4681-88A5-C08F198EFF87}" name="Tiempo dedicado (h)" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{1089505E-D1F6-49DF-BAB1-9822A7A38FB6}" name="Lugar de realización" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -943,13 +949,13 @@
       <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B3" s="9"/>
@@ -958,13 +964,13 @@
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="N5" s="8" t="s">
@@ -1098,14 +1104,44 @@
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="11"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
+      <c r="B12" s="2">
+        <v>46126</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D12" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="11"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
+      <c r="B13" s="2">
+        <v>46126</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D13" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" s="11"/>
@@ -1334,13 +1370,13 @@
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B3" s="4"/>
@@ -1349,13 +1385,13 @@
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="N5" s="1" t="s">
@@ -1489,14 +1525,44 @@
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="2"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
+      <c r="B12" s="2">
+        <v>46126</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D12" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="2"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
+      <c r="B13" s="2">
+        <v>46126</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D13" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
@@ -1725,13 +1791,13 @@
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B3" s="4"/>
@@ -1740,13 +1806,13 @@
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="N5" s="1" t="s">
@@ -1880,14 +1946,44 @@
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="2"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
+      <c r="B12" s="2">
+        <v>46126</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D12" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="2"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
+      <c r="B13" s="2">
+        <v>46126</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D13" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>

</xml_diff>

<commit_message>
Registro de asistencia día 15
</commit_message>
<xml_diff>
--- a/registro_estancias.xlsx
+++ b/registro_estancias.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frang\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferna\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA3D0088-DEE6-4554-B840-9FF23B022262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08775D1-C268-4A51-B27B-44694A1D7B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-15" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nombre1" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="31">
   <si>
     <t>Alumno/a:</t>
   </si>
@@ -119,6 +119,18 @@
   </si>
   <si>
     <t>Gastar intentos de la IA, juntando algunos</t>
+  </si>
+  <si>
+    <t>5:45h</t>
+  </si>
+  <si>
+    <t>Seguir avanzando con fondos del video y revisión de los puntos historicos relevantes del guión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gasto de creditos IA </t>
+  </si>
+  <si>
+    <t>2:00h</t>
   </si>
 </sst>
 </file>
@@ -275,7 +287,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -290,6 +302,18 @@
     <xf numFmtId="14" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -302,18 +326,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="20" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Énfasis1" xfId="2" builtinId="29"/>
@@ -321,65 +334,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="22">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -588,6 +542,65 @@
         <scheme val="minor"/>
       </font>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -602,45 +615,45 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0BDF8D52-2453-4F9C-ACB9-A42D249CFCDF}" name="Fecha" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{04B31198-F76D-4FF5-9268-5FDFE4ECEBE2}" name="Hora inicio" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{DDD0E146-15E7-4D7C-B06E-B38DE0296A38}" name="Hora fin" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{F1A9F247-B63D-4C25-9111-14F13A0959C9}" name="Tareas realizadas" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{32907A34-0575-4F46-A5D0-8BFC39ACFB84}" name="Tiempo dedicado (h)" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{A6ABF540-9F00-4B21-9CD1-F5694FC959C9}" name="Lugar de realización" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{0BDF8D52-2453-4F9C-ACB9-A42D249CFCDF}" name="Fecha" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{04B31198-F76D-4FF5-9268-5FDFE4ECEBE2}" name="Hora inicio" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{DDD0E146-15E7-4D7C-B06E-B38DE0296A38}" name="Hora fin" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{F1A9F247-B63D-4C25-9111-14F13A0959C9}" name="Tareas realizadas" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{32907A34-0575-4F46-A5D0-8BFC39ACFB84}" name="Tiempo dedicado (h)" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{A6ABF540-9F00-4B21-9CD1-F5694FC959C9}" name="Lugar de realización" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="13" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{6717099B-BCF7-48F1-8C12-2FB104043E34}" name="Fecha" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{62A61D49-49F7-40AD-B517-D821200346E1}" name="Hora inicio" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{0EC89713-22B4-4357-96FB-DDBA8AAFD4E2}" name="Hora fin" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{1535F3D9-2D46-4B00-AC9D-A3B5A1FAE726}" name="Tareas realizadas" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{5C84EBA8-F84D-40E8-8B50-A63C5489A5D3}" name="Tiempo dedicado (h)" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{A113B472-3061-44DC-830B-0CB7CF97CD1F}" name="Lugar de realización" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{6717099B-BCF7-48F1-8C12-2FB104043E34}" name="Fecha" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{62A61D49-49F7-40AD-B517-D821200346E1}" name="Hora inicio" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{0EC89713-22B4-4357-96FB-DDBA8AAFD4E2}" name="Hora fin" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{1535F3D9-2D46-4B00-AC9D-A3B5A1FAE726}" name="Tareas realizadas" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{5C84EBA8-F84D-40E8-8B50-A63C5489A5D3}" name="Tiempo dedicado (h)" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{A113B472-3061-44DC-830B-0CB7CF97CD1F}" name="Lugar de realización" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="21" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{08C5D867-C4F7-42FE-B57C-F663CFF2AF17}" name="Fecha" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{C94CC689-C9E6-48B0-9B66-144C47C374AC}" name="Hora inicio" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{257A2ACB-E90D-4206-9538-AE9CCA80B025}" name="Hora fin" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{D70305DF-1893-438D-A18F-E5A3143BA874}" name="Tareas realizadas" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{C97A83D8-08D8-4681-88A5-C08F198EFF87}" name="Tiempo dedicado (h)" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{1089505E-D1F6-49DF-BAB1-9822A7A38FB6}" name="Lugar de realización" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{08C5D867-C4F7-42FE-B57C-F663CFF2AF17}" name="Fecha" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{C94CC689-C9E6-48B0-9B66-144C47C374AC}" name="Hora inicio" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{257A2ACB-E90D-4206-9538-AE9CCA80B025}" name="Hora fin" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{D70305DF-1893-438D-A18F-E5A3143BA874}" name="Tareas realizadas" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{C97A83D8-08D8-4681-88A5-C08F198EFF87}" name="Tiempo dedicado (h)" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{1089505E-D1F6-49DF-BAB1-9822A7A38FB6}" name="Lugar de realización" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -932,52 +945,52 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB0F8AD9-C14E-4D3B-B863-349590932F56}">
   <dimension ref="B2:N51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" style="8" customWidth="1"/>
     <col min="2" max="4" width="15" style="8" customWidth="1"/>
     <col min="5" max="5" width="40" style="8" customWidth="1"/>
     <col min="6" max="6" width="20" style="8" customWidth="1"/>
-    <col min="7" max="7" width="24.33203125" style="8" customWidth="1"/>
-    <col min="8" max="8" width="48.44140625" style="8" customWidth="1"/>
-    <col min="9" max="13" width="8.88671875" style="8"/>
-    <col min="14" max="14" width="8.88671875" style="8" hidden="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="8"/>
+    <col min="7" max="7" width="24.28515625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="48.42578125" style="8" customWidth="1"/>
+    <col min="9" max="13" width="8.85546875" style="8"/>
+    <col min="14" max="14" width="8.85546875" style="8" hidden="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.85546875" style="8"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-    </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="9"/>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-    </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="8" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B6" s="10" t="s">
         <v>3</v>
       </c>
@@ -1000,7 +1013,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
         <v>46121</v>
       </c>
@@ -1023,7 +1036,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
         <v>46121</v>
       </c>
@@ -1043,7 +1056,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
         <v>46122</v>
       </c>
@@ -1063,7 +1076,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>46125</v>
       </c>
@@ -1083,7 +1096,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>46125</v>
       </c>
@@ -1103,7 +1116,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="2">
         <v>46126</v>
       </c>
@@ -1123,7 +1136,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B13" s="2">
         <v>46126</v>
       </c>
@@ -1143,192 +1156,222 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B14" s="11"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B15" s="11"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B14" s="2">
+        <v>46127</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D14" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B15" s="2">
+        <v>46127</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D15" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16" s="11"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="11"/>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="11"/>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="11"/>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="11"/>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="11"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="11"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="11"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="11"/>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25" s="11"/>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B26" s="11"/>
       <c r="C26" s="12"/>
       <c r="D26" s="12"/>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B27" s="11"/>
       <c r="C27" s="12"/>
       <c r="D27" s="12"/>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B28" s="11"/>
       <c r="C28" s="12"/>
       <c r="D28" s="12"/>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="11"/>
       <c r="C29" s="12"/>
       <c r="D29" s="12"/>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="11"/>
       <c r="C30" s="12"/>
       <c r="D30" s="12"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="11"/>
       <c r="C31" s="12"/>
       <c r="D31" s="12"/>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B32" s="11"/>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" s="11"/>
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" s="11"/>
       <c r="C34" s="12"/>
       <c r="D34" s="12"/>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" s="11"/>
       <c r="C35" s="12"/>
       <c r="D35" s="12"/>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="11"/>
       <c r="C36" s="12"/>
       <c r="D36" s="12"/>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="11"/>
       <c r="C37" s="12"/>
       <c r="D37" s="12"/>
     </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" s="11"/>
       <c r="C38" s="12"/>
       <c r="D38" s="12"/>
     </row>
-    <row r="39" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B39" s="11"/>
       <c r="C39" s="12"/>
       <c r="D39" s="12"/>
     </row>
-    <row r="40" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B40" s="11"/>
       <c r="C40" s="12"/>
       <c r="D40" s="12"/>
     </row>
-    <row r="41" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B41" s="11"/>
       <c r="C41" s="12"/>
       <c r="D41" s="12"/>
     </row>
-    <row r="42" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="11"/>
       <c r="C42" s="12"/>
       <c r="D42" s="12"/>
     </row>
-    <row r="43" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="11"/>
       <c r="C43" s="12"/>
       <c r="D43" s="12"/>
     </row>
-    <row r="44" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="11"/>
       <c r="C44" s="12"/>
       <c r="D44" s="12"/>
     </row>
-    <row r="45" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" s="11"/>
       <c r="C45" s="12"/>
       <c r="D45" s="12"/>
     </row>
-    <row r="46" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B46" s="11"/>
       <c r="C46" s="12"/>
       <c r="D46" s="12"/>
     </row>
-    <row r="47" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B47" s="11"/>
       <c r="C47" s="12"/>
       <c r="D47" s="12"/>
     </row>
-    <row r="48" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B48" s="11"/>
       <c r="C48" s="12"/>
       <c r="D48" s="12"/>
     </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B49" s="11"/>
       <c r="C49" s="12"/>
       <c r="D49" s="12"/>
     </row>
-    <row r="50" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B50" s="11"/>
       <c r="C50" s="12"/>
       <c r="D50" s="12"/>
     </row>
-    <row r="51" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B51" s="11"/>
       <c r="C51" s="12"/>
       <c r="D51" s="12"/>
@@ -1353,52 +1396,52 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:N51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" style="1" customWidth="1"/>
     <col min="2" max="4" width="15" style="1" customWidth="1"/>
     <col min="5" max="5" width="40" style="1" customWidth="1"/>
     <col min="6" max="6" width="20" style="1" customWidth="1"/>
-    <col min="7" max="7" width="24.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="48.44140625" style="1" customWidth="1"/>
-    <col min="9" max="13" width="8.88671875" style="1"/>
-    <col min="14" max="14" width="8.88671875" style="1" hidden="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="1"/>
+    <col min="7" max="7" width="24.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="48.42578125" style="1" customWidth="1"/>
+    <col min="9" max="13" width="8.85546875" style="1"/>
+    <col min="14" max="14" width="8.85546875" style="1" hidden="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-    </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-    </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1421,7 +1464,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
         <v>46121</v>
       </c>
@@ -1444,7 +1487,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
         <v>46121</v>
       </c>
@@ -1464,7 +1507,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
         <v>46122</v>
       </c>
@@ -1484,7 +1527,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>46125</v>
       </c>
@@ -1504,7 +1547,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>46125</v>
       </c>
@@ -1524,7 +1567,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="2">
         <v>46126</v>
       </c>
@@ -1544,7 +1587,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B13" s="2">
         <v>46126</v>
       </c>
@@ -1564,192 +1607,222 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B14" s="2"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B15" s="2"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B14" s="2">
+        <v>46127</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D14" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B15" s="2">
+        <v>46127</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D15" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="2"/>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="2"/>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="2"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="2"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25" s="2"/>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B26" s="2"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B27" s="2"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B28" s="2"/>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="2"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="2"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="2"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B32" s="2"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" s="2"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" s="2"/>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" s="2"/>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="2"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="2"/>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
     </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" s="2"/>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
     </row>
-    <row r="39" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B39" s="2"/>
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
     </row>
-    <row r="40" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B40" s="2"/>
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
     </row>
-    <row r="41" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B41" s="2"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
     </row>
-    <row r="42" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="2"/>
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
     </row>
-    <row r="43" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="2"/>
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
     </row>
-    <row r="44" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="2"/>
       <c r="C44" s="6"/>
       <c r="D44" s="6"/>
     </row>
-    <row r="45" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" s="2"/>
       <c r="C45" s="6"/>
       <c r="D45" s="6"/>
     </row>
-    <row r="46" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B46" s="2"/>
       <c r="C46" s="6"/>
       <c r="D46" s="6"/>
     </row>
-    <row r="47" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B47" s="2"/>
       <c r="C47" s="6"/>
       <c r="D47" s="6"/>
     </row>
-    <row r="48" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B48" s="2"/>
       <c r="C48" s="6"/>
       <c r="D48" s="6"/>
     </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B49" s="2"/>
       <c r="C49" s="6"/>
       <c r="D49" s="6"/>
     </row>
-    <row r="50" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B50" s="2"/>
       <c r="C50" s="6"/>
       <c r="D50" s="6"/>
     </row>
-    <row r="51" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B51" s="2"/>
       <c r="C51" s="6"/>
       <c r="D51" s="6"/>
@@ -1774,52 +1847,52 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3CBE6F9-F18B-4FF1-9154-4A49880368D0}">
   <dimension ref="B2:N51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" style="1" customWidth="1"/>
     <col min="2" max="4" width="15" style="1" customWidth="1"/>
     <col min="5" max="5" width="40" style="1" customWidth="1"/>
     <col min="6" max="6" width="20" style="1" customWidth="1"/>
-    <col min="7" max="7" width="24.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="48.44140625" style="1" customWidth="1"/>
-    <col min="9" max="13" width="8.88671875" style="1"/>
-    <col min="14" max="14" width="8.88671875" style="1" hidden="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="1"/>
+    <col min="7" max="7" width="24.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="48.42578125" style="1" customWidth="1"/>
+    <col min="9" max="13" width="8.85546875" style="1"/>
+    <col min="14" max="14" width="8.85546875" style="1" hidden="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-    </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-    </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1842,7 +1915,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
         <v>46121</v>
       </c>
@@ -1865,7 +1938,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
         <v>46121</v>
       </c>
@@ -1885,7 +1958,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
         <v>46122</v>
       </c>
@@ -1905,7 +1978,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>46125</v>
       </c>
@@ -1925,7 +1998,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>46125</v>
       </c>
@@ -1945,7 +2018,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="2">
         <v>46126</v>
       </c>
@@ -1965,7 +2038,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B13" s="2">
         <v>46126</v>
       </c>
@@ -1985,192 +2058,222 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B14" s="2"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B15" s="2"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B14" s="11">
+        <v>46127</v>
+      </c>
+      <c r="C14" s="12">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D14" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B15" s="11">
+        <v>46127</v>
+      </c>
+      <c r="C15" s="12">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D15" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="2"/>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="2"/>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="2"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="2"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25" s="2"/>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B26" s="2"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B27" s="2"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B28" s="2"/>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="2"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="2"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="2"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B32" s="2"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" s="2"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" s="2"/>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" s="2"/>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="2"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="2"/>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
     </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" s="2"/>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
     </row>
-    <row r="39" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B39" s="2"/>
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
     </row>
-    <row r="40" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B40" s="2"/>
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
     </row>
-    <row r="41" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B41" s="2"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
     </row>
-    <row r="42" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="2"/>
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
     </row>
-    <row r="43" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="2"/>
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
     </row>
-    <row r="44" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="2"/>
       <c r="C44" s="6"/>
       <c r="D44" s="6"/>
     </row>
-    <row r="45" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" s="2"/>
       <c r="C45" s="6"/>
       <c r="D45" s="6"/>
     </row>
-    <row r="46" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B46" s="2"/>
       <c r="C46" s="6"/>
       <c r="D46" s="6"/>
     </row>
-    <row r="47" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B47" s="2"/>
       <c r="C47" s="6"/>
       <c r="D47" s="6"/>
     </row>
-    <row r="48" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B48" s="2"/>
       <c r="C48" s="6"/>
       <c r="D48" s="6"/>
     </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B49" s="2"/>
       <c r="C49" s="6"/>
       <c r="D49" s="6"/>
     </row>
-    <row r="50" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B50" s="2"/>
       <c r="C50" s="6"/>
       <c r="D50" s="6"/>
     </row>
-    <row r="51" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B51" s="2"/>
       <c r="C51" s="6"/>
       <c r="D51" s="6"/>

</xml_diff>

<commit_message>
Registro de estancias día 16
</commit_message>
<xml_diff>
--- a/registro_estancias.xlsx
+++ b/registro_estancias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferna\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08775D1-C268-4A51-B27B-44694A1D7B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44F58B53-034E-4BEC-8ED6-FABC7394B95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-15" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nombre1" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="34">
   <si>
     <t>Alumno/a:</t>
   </si>
@@ -131,6 +131,15 @@
   </si>
   <si>
     <t>2:00h</t>
+  </si>
+  <si>
+    <t>Hacemos nuevos videos y arreglamos detalles5:45h</t>
+  </si>
+  <si>
+    <t>Gastamos creditos de flow y edición de dialogos</t>
+  </si>
+  <si>
+    <t>2h</t>
   </si>
 </sst>
 </file>
@@ -302,6 +311,7 @@
     <xf numFmtId="14" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="20" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -326,7 +336,6 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Énfasis1" xfId="2" builtinId="29"/>
@@ -962,13 +971,13 @@
       <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="9"/>
@@ -977,13 +986,13 @@
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="8" t="s">
@@ -1197,86 +1206,114 @@
       </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="11"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="11"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="2">
+        <v>46128</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D16" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="2">
+        <v>46128</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D17" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="11"/>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="11"/>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="11"/>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="11"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="11"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="11"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="11"/>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="11"/>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="11"/>
       <c r="C26" s="12"/>
       <c r="D26" s="12"/>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" s="11"/>
       <c r="C27" s="12"/>
       <c r="D27" s="12"/>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B28" s="11"/>
       <c r="C28" s="12"/>
       <c r="D28" s="12"/>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" s="11"/>
       <c r="C29" s="12"/>
       <c r="D29" s="12"/>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" s="11"/>
       <c r="C30" s="12"/>
       <c r="D30" s="12"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="11"/>
       <c r="C31" s="12"/>
       <c r="D31" s="12"/>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="11"/>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
@@ -1413,13 +1450,13 @@
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -1428,13 +1465,13 @@
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="1" t="s">
@@ -1648,86 +1685,113 @@
       </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="2"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="2"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="2">
+        <v>46128</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D16" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="2">
+        <v>46128</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D17" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="2"/>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="2"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="2"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="2"/>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="2"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" s="2"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B28" s="2"/>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" s="2"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" s="2"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="2"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="2"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
@@ -1864,13 +1928,13 @@
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -1879,13 +1943,13 @@
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="1" t="s">
@@ -2071,7 +2135,7 @@
       <c r="E14" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F14" s="22" t="s">
+      <c r="F14" s="14" t="s">
         <v>27</v>
       </c>
       <c r="G14" s="8" t="s">
@@ -2099,86 +2163,113 @@
       </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="2"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="2"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="2">
+        <v>46128</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D16" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="2">
+        <v>46128</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D17" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="2"/>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="2"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="2"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="2"/>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="2"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" s="2"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B28" s="2"/>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" s="2"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" s="2"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="2"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="2"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>

</xml_diff>

<commit_message>
Registro de estancias día 20
</commit_message>
<xml_diff>
--- a/registro_estancias.xlsx
+++ b/registro_estancias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferna\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44F58B53-034E-4BEC-8ED6-FABC7394B95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{525F1A73-0D0F-4E0D-A39B-AE0E4B6AF20A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nombre1" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="36">
   <si>
     <t>Alumno/a:</t>
   </si>
@@ -140,6 +140,12 @@
   </si>
   <si>
     <t>2h</t>
+  </si>
+  <si>
+    <t>Comenzamos a avanzar con los dialogos del personaje pricipal del video</t>
+  </si>
+  <si>
+    <t>Gasto creditos IA</t>
   </si>
 </sst>
 </file>
@@ -312,18 +318,6 @@
     <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="20" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -336,6 +330,18 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Énfasis1" xfId="2" builtinId="29"/>
@@ -343,6 +349,65 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="22">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -551,65 +616,6 @@
         <scheme val="minor"/>
       </font>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -624,45 +630,45 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0BDF8D52-2453-4F9C-ACB9-A42D249CFCDF}" name="Fecha" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{04B31198-F76D-4FF5-9268-5FDFE4ECEBE2}" name="Hora inicio" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{DDD0E146-15E7-4D7C-B06E-B38DE0296A38}" name="Hora fin" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{F1A9F247-B63D-4C25-9111-14F13A0959C9}" name="Tareas realizadas" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{32907A34-0575-4F46-A5D0-8BFC39ACFB84}" name="Tiempo dedicado (h)" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{A6ABF540-9F00-4B21-9CD1-F5694FC959C9}" name="Lugar de realización" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{0BDF8D52-2453-4F9C-ACB9-A42D249CFCDF}" name="Fecha" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{04B31198-F76D-4FF5-9268-5FDFE4ECEBE2}" name="Hora inicio" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{DDD0E146-15E7-4D7C-B06E-B38DE0296A38}" name="Hora fin" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{F1A9F247-B63D-4C25-9111-14F13A0959C9}" name="Tareas realizadas" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{32907A34-0575-4F46-A5D0-8BFC39ACFB84}" name="Tiempo dedicado (h)" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{A6ABF540-9F00-4B21-9CD1-F5694FC959C9}" name="Lugar de realización" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="13" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{6717099B-BCF7-48F1-8C12-2FB104043E34}" name="Fecha" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{62A61D49-49F7-40AD-B517-D821200346E1}" name="Hora inicio" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{0EC89713-22B4-4357-96FB-DDBA8AAFD4E2}" name="Hora fin" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{1535F3D9-2D46-4B00-AC9D-A3B5A1FAE726}" name="Tareas realizadas" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{5C84EBA8-F84D-40E8-8B50-A63C5489A5D3}" name="Tiempo dedicado (h)" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{A113B472-3061-44DC-830B-0CB7CF97CD1F}" name="Lugar de realización" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{6717099B-BCF7-48F1-8C12-2FB104043E34}" name="Fecha" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{62A61D49-49F7-40AD-B517-D821200346E1}" name="Hora inicio" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{0EC89713-22B4-4357-96FB-DDBA8AAFD4E2}" name="Hora fin" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{1535F3D9-2D46-4B00-AC9D-A3B5A1FAE726}" name="Tareas realizadas" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{5C84EBA8-F84D-40E8-8B50-A63C5489A5D3}" name="Tiempo dedicado (h)" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{A113B472-3061-44DC-830B-0CB7CF97CD1F}" name="Lugar de realización" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="21" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{08C5D867-C4F7-42FE-B57C-F663CFF2AF17}" name="Fecha" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{C94CC689-C9E6-48B0-9B66-144C47C374AC}" name="Hora inicio" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{257A2ACB-E90D-4206-9538-AE9CCA80B025}" name="Hora fin" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{D70305DF-1893-438D-A18F-E5A3143BA874}" name="Tareas realizadas" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{C97A83D8-08D8-4681-88A5-C08F198EFF87}" name="Tiempo dedicado (h)" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{1089505E-D1F6-49DF-BAB1-9822A7A38FB6}" name="Lugar de realización" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{08C5D867-C4F7-42FE-B57C-F663CFF2AF17}" name="Fecha" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{C94CC689-C9E6-48B0-9B66-144C47C374AC}" name="Hora inicio" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{257A2ACB-E90D-4206-9538-AE9CCA80B025}" name="Hora fin" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{D70305DF-1893-438D-A18F-E5A3143BA874}" name="Tareas realizadas" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{C97A83D8-08D8-4681-88A5-C08F198EFF87}" name="Tiempo dedicado (h)" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{1089505E-D1F6-49DF-BAB1-9822A7A38FB6}" name="Lugar de realización" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -971,13 +977,13 @@
       <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="9"/>
@@ -986,13 +992,13 @@
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="8" t="s">
@@ -1244,14 +1250,44 @@
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="11"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
+      <c r="B18" s="11">
+        <v>46132</v>
+      </c>
+      <c r="C18" s="12">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D18" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B19" s="11"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
+      <c r="B19" s="11">
+        <v>46132</v>
+      </c>
+      <c r="C19" s="12">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D19" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="11"/>
@@ -1450,13 +1486,13 @@
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -1465,13 +1501,13 @@
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="1" t="s">
@@ -1722,14 +1758,44 @@
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="2"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
+      <c r="B18" s="11">
+        <v>46132</v>
+      </c>
+      <c r="C18" s="12">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D18" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B19" s="2"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
+      <c r="B19" s="11">
+        <v>46132</v>
+      </c>
+      <c r="C19" s="12">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D19" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
@@ -1928,13 +1994,13 @@
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -1943,13 +2009,13 @@
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="1" t="s">
@@ -2200,14 +2266,44 @@
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="2"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
+      <c r="B18" s="11">
+        <v>46132</v>
+      </c>
+      <c r="C18" s="12">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D18" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B19" s="2"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
+      <c r="B19" s="11">
+        <v>46132</v>
+      </c>
+      <c r="C19" s="12">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D19" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>

</xml_diff>

<commit_message>
Registro estancias día 21
</commit_message>
<xml_diff>
--- a/registro_estancias.xlsx
+++ b/registro_estancias.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferna\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAM Virtual\Estancias Formativas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{525F1A73-0D0F-4E0D-A39B-AE0E4B6AF20A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BC53E64-9957-445A-BE43-2B2F57B3197B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-15" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nombre1" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="37">
   <si>
     <t>Alumno/a:</t>
   </si>
@@ -146,6 +146,9 @@
   </si>
   <si>
     <t>Gasto creditos IA</t>
+  </si>
+  <si>
+    <t>Introducimos parte de dialogos del personaje5:45h</t>
   </si>
 </sst>
 </file>
@@ -318,6 +321,18 @@
     <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="20" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -330,18 +345,6 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Énfasis1" xfId="2" builtinId="29"/>
@@ -349,65 +352,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="22">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -616,6 +560,65 @@
         <scheme val="minor"/>
       </font>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -630,45 +633,45 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{251D8C2D-F7F1-4A24-8F41-6AC60ADCDF37}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0BDF8D52-2453-4F9C-ACB9-A42D249CFCDF}" name="Fecha" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{04B31198-F76D-4FF5-9268-5FDFE4ECEBE2}" name="Hora inicio" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{DDD0E146-15E7-4D7C-B06E-B38DE0296A38}" name="Hora fin" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{F1A9F247-B63D-4C25-9111-14F13A0959C9}" name="Tareas realizadas" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{32907A34-0575-4F46-A5D0-8BFC39ACFB84}" name="Tiempo dedicado (h)" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{A6ABF540-9F00-4B21-9CD1-F5694FC959C9}" name="Lugar de realización" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{0BDF8D52-2453-4F9C-ACB9-A42D249CFCDF}" name="Fecha" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{04B31198-F76D-4FF5-9268-5FDFE4ECEBE2}" name="Hora inicio" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{DDD0E146-15E7-4D7C-B06E-B38DE0296A38}" name="Hora fin" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{F1A9F247-B63D-4C25-9111-14F13A0959C9}" name="Tareas realizadas" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{32907A34-0575-4F46-A5D0-8BFC39ACFB84}" name="Tiempo dedicado (h)" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{A6ABF540-9F00-4B21-9CD1-F5694FC959C9}" name="Lugar de realización" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="13" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{ADC44A1E-9C8E-4751-B277-34DEB252ECA4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{6717099B-BCF7-48F1-8C12-2FB104043E34}" name="Fecha" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{62A61D49-49F7-40AD-B517-D821200346E1}" name="Hora inicio" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{0EC89713-22B4-4357-96FB-DDBA8AAFD4E2}" name="Hora fin" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{1535F3D9-2D46-4B00-AC9D-A3B5A1FAE726}" name="Tareas realizadas" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{5C84EBA8-F84D-40E8-8B50-A63C5489A5D3}" name="Tiempo dedicado (h)" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{A113B472-3061-44DC-830B-0CB7CF97CD1F}" name="Lugar de realización" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{6717099B-BCF7-48F1-8C12-2FB104043E34}" name="Fecha" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{62A61D49-49F7-40AD-B517-D821200346E1}" name="Hora inicio" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{0EC89713-22B4-4357-96FB-DDBA8AAFD4E2}" name="Hora fin" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{1535F3D9-2D46-4B00-AC9D-A3B5A1FAE726}" name="Tareas realizadas" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{5C84EBA8-F84D-40E8-8B50-A63C5489A5D3}" name="Tiempo dedicado (h)" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{A113B472-3061-44DC-830B-0CB7CF97CD1F}" name="Lugar de realización" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="21" headerRowCellStyle="Énfasis1">
   <autoFilter ref="B6:G51" xr:uid="{AE84FB71-BB8B-4A55-BEAB-6A0390B3B9D2}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{08C5D867-C4F7-42FE-B57C-F663CFF2AF17}" name="Fecha" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{C94CC689-C9E6-48B0-9B66-144C47C374AC}" name="Hora inicio" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{257A2ACB-E90D-4206-9538-AE9CCA80B025}" name="Hora fin" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{D70305DF-1893-438D-A18F-E5A3143BA874}" name="Tareas realizadas" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{C97A83D8-08D8-4681-88A5-C08F198EFF87}" name="Tiempo dedicado (h)" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{1089505E-D1F6-49DF-BAB1-9822A7A38FB6}" name="Lugar de realización" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{08C5D867-C4F7-42FE-B57C-F663CFF2AF17}" name="Fecha" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{C94CC689-C9E6-48B0-9B66-144C47C374AC}" name="Hora inicio" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{257A2ACB-E90D-4206-9538-AE9CCA80B025}" name="Hora fin" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{D70305DF-1893-438D-A18F-E5A3143BA874}" name="Tareas realizadas" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{C97A83D8-08D8-4681-88A5-C08F198EFF87}" name="Tiempo dedicado (h)" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{1089505E-D1F6-49DF-BAB1-9822A7A38FB6}" name="Lugar de realización" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -977,13 +980,13 @@
       <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="9"/>
@@ -992,13 +995,13 @@
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="8" t="s">
@@ -1290,24 +1293,58 @@
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B20" s="11"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
+      <c r="B20" s="2">
+        <v>46133</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D20" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="11"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
+      <c r="B21" s="2">
+        <v>46133</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D21" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B22" s="11"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B23" s="11"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="11"/>
@@ -1486,13 +1523,13 @@
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -1501,13 +1538,13 @@
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="1" t="s">
@@ -1798,14 +1835,41 @@
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B20" s="2"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
+      <c r="B20" s="2">
+        <v>46133</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D20" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="2"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
+      <c r="B21" s="2">
+        <v>46133</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D21" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>
@@ -1994,13 +2058,13 @@
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -2009,13 +2073,13 @@
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N5" s="1" t="s">
@@ -2306,14 +2370,41 @@
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B20" s="2"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
+      <c r="B20" s="2">
+        <v>46133</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D20" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="2"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
+      <c r="B21" s="2">
+        <v>46133</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D21" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>

</xml_diff>

<commit_message>
Registro de estancias día 22
</commit_message>
<xml_diff>
--- a/registro_estancias.xlsx
+++ b/registro_estancias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAM Virtual\Estancias Formativas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BC53E64-9957-445A-BE43-2B2F57B3197B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B244CE4-1EC6-4C2B-885E-5807D379BAB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-15" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nombre1" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="38">
   <si>
     <t>Alumno/a:</t>
   </si>
@@ -149,6 +149,9 @@
   </si>
   <si>
     <t>Introducimos parte de dialogos del personaje5:45h</t>
+  </si>
+  <si>
+    <t>Introducimos dialogos del personaje</t>
   </si>
 </sst>
 </file>
@@ -1331,20 +1334,44 @@
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B22" s="2"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
+      <c r="B22" s="2">
+        <v>46134</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D22" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B23" s="2"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
+      <c r="B23" s="2">
+        <v>46134</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D23" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="11"/>
@@ -1872,14 +1899,44 @@
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B22" s="2"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
+      <c r="B22" s="2">
+        <v>46134</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D22" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B23" s="2"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
+      <c r="B23" s="2">
+        <v>46134</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D23" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="2"/>
@@ -2407,14 +2464,44 @@
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B22" s="2"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
+      <c r="B22" s="2">
+        <v>46134</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D22" s="6">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B23" s="2"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
+      <c r="B23" s="2">
+        <v>46134</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D23" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="2"/>

</xml_diff>